<commit_message>
Persistence added to CCI page, alpha edition
</commit_message>
<xml_diff>
--- a/data/sdlc_macro.xlsx
+++ b/data/sdlc_macro.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wangc/projects/SHIELDS/BAHAMAS/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://inl-my.sharepoint.com/personal/edward_chen_inl_gov/Documents/Projects/RISA/BAHAMAS/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B93F141-2777-D745-A7B7-53F5A15901A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{4B93F141-2777-D745-A7B7-53F5A15901A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AB243238-5FCE-4D1E-9895-C36C1F522598}"/>
   <bookViews>
-    <workbookView xWindow="320" yWindow="820" windowWidth="34560" windowHeight="21100" activeTab="5" xr2:uid="{1CBAA6C8-6300-440C-AE44-018A87B8EEBB}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" activeTab="5" xr2:uid="{1CBAA6C8-6300-440C-AE44-018A87B8EEBB}"/>
   </bookViews>
   <sheets>
     <sheet name="Concept" sheetId="8" r:id="rId1"/>
@@ -437,15 +437,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{737D0550-1A36-42FD-907A-05CC337EE242}">
   <dimension ref="A1:D2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.6640625" customWidth="1"/>
-    <col min="2" max="2" width="24.5" customWidth="1"/>
-    <col min="3" max="3" width="16.1640625" customWidth="1"/>
-    <col min="4" max="4" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.7109375" customWidth="1"/>
+    <col min="2" max="2" width="24.42578125" customWidth="1"/>
+    <col min="3" max="3" width="16.140625" customWidth="1"/>
+    <col min="4" max="4" width="14.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -459,7 +459,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>0.25</v>
       </c>
@@ -481,16 +481,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3AFAD734-E067-4CA0-BDBA-F4AC1A4E2B2B}">
   <dimension ref="A1:D2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="28.33203125" customWidth="1"/>
-    <col min="2" max="2" width="25.33203125" customWidth="1"/>
-    <col min="3" max="3" width="47.83203125" customWidth="1"/>
+    <col min="1" max="1" width="28.28515625" customWidth="1"/>
+    <col min="2" max="2" width="25.28515625" customWidth="1"/>
+    <col min="3" max="3" width="47.85546875" customWidth="1"/>
     <col min="4" max="4" width="16" customWidth="1"/>
-    <col min="5" max="5" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -504,7 +504,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>0.25</v>
       </c>
@@ -527,16 +527,16 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C83E50E1-7FF6-47C0-B2D3-965E93D78F83}">
   <dimension ref="A1:D12"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="28.1640625" customWidth="1"/>
-    <col min="2" max="2" width="28.5" customWidth="1"/>
+    <col min="1" max="1" width="28.140625" customWidth="1"/>
+    <col min="2" max="2" width="28.42578125" customWidth="1"/>
     <col min="3" max="3" width="81" customWidth="1"/>
-    <col min="4" max="4" width="13.33203125" customWidth="1"/>
-    <col min="5" max="5" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.28515625" customWidth="1"/>
+    <col min="5" max="5" width="14.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -550,7 +550,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>0.25</v>
       </c>
@@ -564,16 +564,16 @@
         <v>0.96</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C3" s="2"/>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C6" s="1"/>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C11" s="1"/>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C12" s="1"/>
     </row>
   </sheetData>
@@ -585,16 +585,16 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B5B5E32-C01B-4578-9E30-68F8F8C93AA7}">
   <dimension ref="A1:D2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="28.33203125" customWidth="1"/>
-    <col min="2" max="2" width="26.1640625" customWidth="1"/>
+    <col min="1" max="1" width="28.28515625" customWidth="1"/>
+    <col min="2" max="2" width="26.140625" customWidth="1"/>
     <col min="3" max="3" width="46" customWidth="1"/>
-    <col min="4" max="4" width="13.6640625" customWidth="1"/>
-    <col min="5" max="5" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.7109375" customWidth="1"/>
+    <col min="5" max="5" width="14.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -608,7 +608,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>0.25</v>
       </c>
@@ -630,16 +630,16 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D51F2905-0C23-4BBC-9AE6-D1498E006EAB}">
   <dimension ref="A1:D2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="25.33203125" customWidth="1"/>
-    <col min="2" max="2" width="23.5" customWidth="1"/>
-    <col min="3" max="3" width="33.83203125" customWidth="1"/>
-    <col min="4" max="4" width="13.83203125" customWidth="1"/>
-    <col min="5" max="5" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.28515625" customWidth="1"/>
+    <col min="2" max="2" width="23.42578125" customWidth="1"/>
+    <col min="3" max="3" width="33.85546875" customWidth="1"/>
+    <col min="4" max="4" width="13.85546875" customWidth="1"/>
+    <col min="5" max="5" width="14.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -653,7 +653,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>0.25</v>
       </c>
@@ -675,16 +675,16 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{53A5414B-10E4-4CE1-A468-21D1AFA5E248}">
   <dimension ref="A1:D2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="25.5" customWidth="1"/>
-    <col min="2" max="2" width="23.33203125" customWidth="1"/>
-    <col min="3" max="3" width="33.1640625" customWidth="1"/>
-    <col min="4" max="4" width="14" customWidth="1"/>
-    <col min="5" max="5" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.42578125" customWidth="1"/>
+    <col min="2" max="2" width="23.28515625" customWidth="1"/>
+    <col min="3" max="3" width="33.140625" customWidth="1"/>
+    <col min="4" max="4" width="22" customWidth="1"/>
+    <col min="5" max="5" width="14.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -698,7 +698,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>0.25</v>
       </c>

</xml_diff>

<commit_message>
Added xlsx files to preliminary, comprehensive, and CCI
</commit_message>
<xml_diff>
--- a/data/sdlc_macro.xlsx
+++ b/data/sdlc_macro.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://inl-my.sharepoint.com/personal/edward_chen_inl_gov/Documents/Projects/RISA/BAHAMAS/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{4B93F141-2777-D745-A7B7-53F5A15901A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AB243238-5FCE-4D1E-9895-C36C1F522598}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{4B93F141-2777-D745-A7B7-53F5A15901A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{42748AE0-458C-4721-A183-F1534BB290F4}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" activeTab="5" xr2:uid="{1CBAA6C8-6300-440C-AE44-018A87B8EEBB}"/>
+    <workbookView xWindow="6880" yWindow="10690" windowWidth="19420" windowHeight="10300" xr2:uid="{1CBAA6C8-6300-440C-AE44-018A87B8EEBB}"/>
   </bookViews>
   <sheets>
     <sheet name="Concept" sheetId="8" r:id="rId1"/>
@@ -678,7 +678,7 @@
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.42578125" customWidth="1"/>
-    <col min="2" max="2" width="23.28515625" customWidth="1"/>
+    <col min="2" max="2" width="31.7109375" customWidth="1"/>
     <col min="3" max="3" width="33.140625" customWidth="1"/>
     <col min="4" max="4" width="22" customWidth="1"/>
     <col min="5" max="5" width="14.7109375" bestFit="1" customWidth="1"/>

</xml_diff>